<commit_message>
Fix Tecos 2026 asistencia
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/asistencia/Tecos 2026.xlsx
+++ b/data/asistencia/Tecos 2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="40">
   <si>
     <t>Reporte de disponibilidad por zona</t>
   </si>
@@ -19,7 +19,7 @@
     <t/>
   </si>
   <si>
-    <t>Juego Inaugural: Caliente vs Tecos</t>
+    <t>Juego Inaugural: Charros vs Tecos</t>
   </si>
   <si>
     <t>ZONA</t>
@@ -88,25 +88,25 @@
     <t>Butaca General</t>
   </si>
   <si>
-    <t>99.80%</t>
+    <t>99.47%</t>
   </si>
   <si>
     <t>Butaca Preferente</t>
   </si>
   <si>
-    <t>99.67%</t>
+    <t>97.69%</t>
   </si>
   <si>
     <t>Especial</t>
   </si>
   <si>
-    <t>26.00%</t>
+    <t>72.00%</t>
   </si>
   <si>
     <t>Gradas</t>
   </si>
   <si>
-    <t>39.75%</t>
+    <t>25.29%</t>
   </si>
   <si>
     <t>Palcos</t>
@@ -115,25 +115,22 @@
     <t>Palcos 1ra</t>
   </si>
   <si>
-    <t>98.15%</t>
+    <t>99.07%</t>
   </si>
   <si>
     <t>Palcos 3ra</t>
   </si>
   <si>
-    <t>SUITE</t>
+    <t>Tecobar</t>
   </si>
   <si>
     <t>0.00%</t>
   </si>
   <si>
-    <t>Tecobar</t>
-  </si>
-  <si>
     <t>TOTALES</t>
   </si>
   <si>
-    <t>61.39%</t>
+    <t>53.99%</t>
   </si>
 </sst>
 </file>
@@ -555,7 +552,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R17"/>
+  <dimension ref="A1:R16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="39" customWidth="1"/>
@@ -699,16 +696,16 @@
         <v>24</v>
       </c>
       <c r="B7" s="6">
-        <v>1003</v>
+        <v>566</v>
       </c>
       <c r="C7" s="6">
-        <v>466</v>
+        <v>322</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>22</v>
       </c>
       <c r="E7" s="6">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="F7" s="6" t="s">
         <v>22</v>
@@ -720,7 +717,7 @@
         <v>22</v>
       </c>
       <c r="I7" s="6">
-        <v>474</v>
+        <v>183</v>
       </c>
       <c r="J7" s="6" t="s">
         <v>22</v>
@@ -734,17 +731,17 @@
       <c r="M7" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="N7" s="6">
-        <v>6</v>
+      <c r="N7" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="O7" s="6" t="s">
         <v>22</v>
       </c>
       <c r="P7" s="6">
-        <v>1001</v>
+        <v>563</v>
       </c>
       <c r="Q7" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R7" s="6" t="s">
         <v>25</v>
@@ -755,16 +752,16 @@
         <v>26</v>
       </c>
       <c r="B8" s="6">
-        <v>604</v>
+        <v>1041</v>
       </c>
       <c r="C8" s="6">
-        <v>217</v>
+        <v>489</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="E8" s="6" t="s">
-        <v>22</v>
+      <c r="E8" s="6">
+        <v>14</v>
       </c>
       <c r="F8" s="6" t="s">
         <v>22</v>
@@ -776,7 +773,7 @@
         <v>22</v>
       </c>
       <c r="I8" s="6">
-        <v>385</v>
+        <v>514</v>
       </c>
       <c r="J8" s="6" t="s">
         <v>22</v>
@@ -797,10 +794,10 @@
         <v>22</v>
       </c>
       <c r="P8" s="6">
-        <v>602</v>
+        <v>1017</v>
       </c>
       <c r="Q8" s="6">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="R8" s="6" t="s">
         <v>27</v>
@@ -820,7 +817,7 @@
         <v>22</v>
       </c>
       <c r="E9" s="6">
-        <v>26</v>
+        <v>68</v>
       </c>
       <c r="F9" s="6" t="s">
         <v>22</v>
@@ -831,8 +828,8 @@
       <c r="H9" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="I9" s="6" t="s">
-        <v>22</v>
+      <c r="I9" s="6">
+        <v>4</v>
       </c>
       <c r="J9" s="6" t="s">
         <v>22</v>
@@ -853,10 +850,10 @@
         <v>22</v>
       </c>
       <c r="P9" s="6">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="Q9" s="6">
-        <v>74</v>
+        <v>28</v>
       </c>
       <c r="R9" s="6" t="s">
         <v>29</v>
@@ -870,13 +867,13 @@
         <v>2800</v>
       </c>
       <c r="C10" s="6">
-        <v>828</v>
+        <v>466</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>22</v>
       </c>
       <c r="E10" s="6">
-        <v>285</v>
+        <v>242</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>22</v>
@@ -909,10 +906,10 @@
         <v>22</v>
       </c>
       <c r="P10" s="6">
-        <v>1113</v>
+        <v>708</v>
       </c>
       <c r="Q10" s="6">
-        <v>1687</v>
+        <v>2092</v>
       </c>
       <c r="R10" s="6" t="s">
         <v>31</v>
@@ -931,8 +928,8 @@
       <c r="D11" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="E11" s="6">
-        <v>16</v>
+      <c r="E11" s="6" t="s">
+        <v>22</v>
       </c>
       <c r="F11" s="6" t="s">
         <v>22</v>
@@ -943,8 +940,8 @@
       <c r="H11" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="I11" s="6" t="s">
-        <v>22</v>
+      <c r="I11" s="6">
+        <v>12</v>
       </c>
       <c r="J11" s="6" t="s">
         <v>22</v>
@@ -959,7 +956,7 @@
         <v>22</v>
       </c>
       <c r="N11" s="6">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="O11" s="6" t="s">
         <v>22</v>
@@ -982,7 +979,7 @@
         <v>108</v>
       </c>
       <c r="C12" s="6">
-        <v>34</v>
+        <v>71</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>22</v>
@@ -1000,7 +997,7 @@
         <v>22</v>
       </c>
       <c r="I12" s="6">
-        <v>72</v>
+        <v>36</v>
       </c>
       <c r="J12" s="6" t="s">
         <v>22</v>
@@ -1021,10 +1018,10 @@
         <v>22</v>
       </c>
       <c r="P12" s="6">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="Q12" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R12" s="6" t="s">
         <v>34</v>
@@ -1038,7 +1035,7 @@
         <v>108</v>
       </c>
       <c r="C13" s="6">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>22</v>
@@ -1056,7 +1053,7 @@
         <v>22</v>
       </c>
       <c r="I13" s="6">
-        <v>72</v>
+        <v>48</v>
       </c>
       <c r="J13" s="6" t="s">
         <v>22</v>
@@ -1077,13 +1074,13 @@
         <v>22</v>
       </c>
       <c r="P13" s="6">
-        <v>108</v>
-      </c>
-      <c r="Q13" s="6" t="s">
-        <v>22</v>
+        <v>107</v>
+      </c>
+      <c r="Q13" s="6">
+        <v>1</v>
       </c>
       <c r="R13" s="6" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
@@ -1091,7 +1088,7 @@
         <v>36</v>
       </c>
       <c r="B14" s="6">
-        <v>20</v>
+        <v>150</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>22</v>
@@ -1136,126 +1133,70 @@
         <v>22</v>
       </c>
       <c r="Q14" s="6">
-        <v>20</v>
+        <v>150</v>
       </c>
       <c r="R14" s="6" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B15" s="6">
-        <v>150</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="G15" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="H15" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="I15" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="J15" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="K15" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="L15" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="M15" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="N15" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="O15" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="P15" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q15" s="6">
-        <v>150</v>
-      </c>
-      <c r="R15" s="6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
+      <c r="B15" s="7">
+        <f>SUM(B6:B14)</f>
+      </c>
+      <c r="C15" s="7">
+        <f>SUM(C6:C14)</f>
+      </c>
+      <c r="D15" s="7">
+        <f>SUM(D6:D14)</f>
+      </c>
+      <c r="E15" s="7">
+        <f>SUM(E6:E14)</f>
+      </c>
+      <c r="F15" s="7">
+        <f>SUM(F6:F14)</f>
+      </c>
+      <c r="G15" s="7">
+        <f>SUM(G6:G14)</f>
+      </c>
+      <c r="H15" s="7">
+        <f>SUM(H6:H14)</f>
+      </c>
+      <c r="I15" s="7">
+        <f>SUM(I6:I14)</f>
+      </c>
+      <c r="J15" s="7">
+        <f>SUM(J6:J14)</f>
+      </c>
+      <c r="K15" s="7">
+        <f>SUM(K6:K14)</f>
+      </c>
+      <c r="L15" s="7">
+        <f>SUM(L6:L14)</f>
+      </c>
+      <c r="M15" s="7">
+        <f>SUM(M6:M14)</f>
+      </c>
+      <c r="N15" s="7">
+        <f>SUM(N6:N14)</f>
+      </c>
+      <c r="O15" s="7">
+        <f>SUM(O6:O14)</f>
+      </c>
+      <c r="P15" s="7">
+        <f>SUM(P6:P14)</f>
+      </c>
+      <c r="Q15" s="7">
+        <f>SUM(Q6:Q14)</f>
+      </c>
+      <c r="R15" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="B16" s="7">
-        <f>SUM(B6:B15)</f>
-      </c>
-      <c r="C16" s="7">
-        <f>SUM(C6:C15)</f>
-      </c>
-      <c r="D16" s="7">
-        <f>SUM(D6:D15)</f>
-      </c>
-      <c r="E16" s="7">
-        <f>SUM(E6:E15)</f>
-      </c>
-      <c r="F16" s="7">
-        <f>SUM(F6:F15)</f>
-      </c>
-      <c r="G16" s="7">
-        <f>SUM(G6:G15)</f>
-      </c>
-      <c r="H16" s="7">
-        <f>SUM(H6:H15)</f>
-      </c>
-      <c r="I16" s="7">
-        <f>SUM(I6:I15)</f>
-      </c>
-      <c r="J16" s="7">
-        <f>SUM(J6:J15)</f>
-      </c>
-      <c r="K16" s="7">
-        <f>SUM(K6:K15)</f>
-      </c>
-      <c r="L16" s="7">
-        <f>SUM(L6:L15)</f>
-      </c>
-      <c r="M16" s="7">
-        <f>SUM(M6:M15)</f>
-      </c>
-      <c r="N16" s="7">
-        <f>SUM(N6:N15)</f>
-      </c>
-      <c r="O16" s="7">
-        <f>SUM(O6:O15)</f>
-      </c>
-      <c r="P16" s="7">
-        <f>SUM(P6:P15)</f>
-      </c>
-      <c r="Q16" s="7">
-        <f>SUM(Q6:Q15)</f>
-      </c>
-      <c r="R16" s="7" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
         <v>1</v>
       </c>
     </row>

</xml_diff>